<commit_message>
Compare the community sheet from a CSV of the columns the comparison reads
nation-data/Countries on Eurth.csv holds the sheet's row number and five columns
(Country, Capital, Area, Population, GDPPC). compare_sheet.py reads it; given an
Excel export of the sheet it rewrites the CSV from it and keeps nothing else.
The comparison workbook has three tabs: the stored columns, Map data and Diff.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/nation-data/Countries on Eurth - differences.xlsx
+++ b/nation-data/Countries on Eurth - differences.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F87"/>
+  <dimension ref="A1:F86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -497,7 +497,7 @@
     <row r="2" ht="45" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>82 values differ across 35 nations. "Sheet row" is the row on the Countries of Eurth tab. Where the map's value is the newer one, type it into the sheet, or take them all at once from the Paste-ready tab.</t>
+          <t>81 values differ across 34 nations. "Sheet row" is the row on the Countries of Eurth tab. Where the map's value is the newer one, type it into the sheet, or take them all at once from the Paste-ready tab.</t>
         </is>
       </c>
     </row>
@@ -1458,776 +1458,752 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="11" t="inlineStr">
-        <is>
-          <t>Manamana</t>
-        </is>
-      </c>
-      <c r="B50" s="8" t="n">
-        <v>59</v>
-      </c>
-      <c r="C50" s="8" t="inlineStr">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Marchyydion</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Area (km2)</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="n">
+        <v>429545.88</v>
+      </c>
+      <c r="E50" s="6" t="n">
+        <v>800000</v>
+      </c>
+      <c r="F50" s="7" t="n">
+        <v>0.8624320177392925</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="n"/>
+      <c r="B51" s="8" t="n"/>
+      <c r="C51" s="8" t="inlineStr">
         <is>
           <t>Population</t>
         </is>
       </c>
-      <c r="D50" s="9" t="n">
-        <v>18361225</v>
-      </c>
-      <c r="E50" s="9" t="n">
-        <v>361225</v>
-      </c>
-      <c r="F50" s="10" t="n">
-        <v>-0.9803267483514853</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>Marchyydion</t>
-        </is>
-      </c>
-      <c r="B51" s="5" t="n">
-        <v>60</v>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
+      <c r="D51" s="9" t="n">
+        <v>13000000</v>
+      </c>
+      <c r="E51" s="9" t="n">
+        <v>39724000</v>
+      </c>
+      <c r="F51" s="10" t="n">
+        <v>2.055692307692308</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Mikochi</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
         <is>
           <t>Area (km2)</t>
         </is>
       </c>
-      <c r="D51" s="6" t="n">
-        <v>429545.88</v>
-      </c>
-      <c r="E51" s="6" t="n">
-        <v>800000</v>
-      </c>
-      <c r="F51" s="7" t="n">
-        <v>0.8624320177392925</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="8" t="n"/>
-      <c r="B52" s="8" t="n"/>
-      <c r="C52" s="8" t="inlineStr">
+      <c r="D52" s="6" t="n">
+        <v>76017</v>
+      </c>
+      <c r="E52" s="6" t="n">
+        <v>192532</v>
+      </c>
+      <c r="F52" s="7" t="n">
+        <v>1.532749253456464</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="n"/>
+      <c r="B53" s="5" t="n"/>
+      <c r="C53" s="5" t="inlineStr">
         <is>
           <t>Population</t>
         </is>
       </c>
-      <c r="D52" s="9" t="n">
-        <v>13000000</v>
-      </c>
-      <c r="E52" s="9" t="n">
-        <v>39724000</v>
-      </c>
-      <c r="F52" s="10" t="n">
-        <v>2.055692307692308</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="4" t="inlineStr">
-        <is>
-          <t>Mikochi</t>
-        </is>
-      </c>
-      <c r="B53" s="5" t="n">
-        <v>64</v>
-      </c>
-      <c r="C53" s="5" t="inlineStr">
+      <c r="D53" s="6" t="n">
+        <v>25287241</v>
+      </c>
+      <c r="E53" s="6" t="n">
+        <v>68291582</v>
+      </c>
+      <c r="F53" s="7" t="n">
+        <v>1.700633967936636</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="n"/>
+      <c r="B54" s="8" t="n"/>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>GDPPC</t>
+        </is>
+      </c>
+      <c r="D54" s="9" t="n">
+        <v>28779</v>
+      </c>
+      <c r="E54" s="9" t="n">
+        <v>38653.89</v>
+      </c>
+      <c r="F54" s="10" t="n">
+        <v>0.3431283227353278</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="11" t="inlineStr">
+        <is>
+          <t>Mitō</t>
+        </is>
+      </c>
+      <c r="B55" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>Population</t>
+        </is>
+      </c>
+      <c r="D55" s="9" t="n">
+        <v>9723000</v>
+      </c>
+      <c r="E55" s="9" t="n">
+        <v>13723000</v>
+      </c>
+      <c r="F55" s="10" t="n">
+        <v>0.4113956597757893</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Orioni</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>70</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
         <is>
           <t>Area (km2)</t>
         </is>
       </c>
-      <c r="D53" s="6" t="n">
-        <v>76017</v>
-      </c>
-      <c r="E53" s="6" t="n">
-        <v>192532</v>
-      </c>
-      <c r="F53" s="7" t="n">
-        <v>1.532749253456464</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="5" t="n"/>
-      <c r="B54" s="5" t="n"/>
-      <c r="C54" s="5" t="inlineStr">
+      <c r="D56" s="6" t="n">
+        <v>1155853</v>
+      </c>
+      <c r="E56" s="6" t="n">
+        <v>1320687</v>
+      </c>
+      <c r="F56" s="7" t="n">
+        <v>0.1426080998189216</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="n"/>
+      <c r="B57" s="8" t="n"/>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>GDPPC</t>
+        </is>
+      </c>
+      <c r="D57" s="9" t="n">
+        <v>46131</v>
+      </c>
+      <c r="E57" s="9" t="n">
+        <v>58297.29</v>
+      </c>
+      <c r="F57" s="10" t="n">
+        <v>0.2637334980815504</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>Pentium</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>71</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>Area (km2)</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="n">
+        <v>87500</v>
+      </c>
+      <c r="E58" s="6" t="n">
+        <v>389287</v>
+      </c>
+      <c r="F58" s="7" t="n">
+        <v>3.448994285714286</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="n"/>
+      <c r="B59" s="8" t="n"/>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>GDPPC</t>
+        </is>
+      </c>
+      <c r="D59" s="9" t="n">
+        <v>21220</v>
+      </c>
+      <c r="E59" s="9" t="n">
+        <v>37542</v>
+      </c>
+      <c r="F59" s="10" t="n">
+        <v>0.7691800188501414</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>Poja</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="n">
+        <v>72</v>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>Area (km2)</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="n">
+        <v>340090</v>
+      </c>
+      <c r="E60" s="6" t="n">
+        <v>504767</v>
+      </c>
+      <c r="F60" s="7" t="n">
+        <v>0.4842159428386604</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="n"/>
+      <c r="B61" s="5" t="n"/>
+      <c r="C61" s="5" t="inlineStr">
         <is>
           <t>Population</t>
         </is>
       </c>
-      <c r="D54" s="6" t="n">
-        <v>25287241</v>
-      </c>
-      <c r="E54" s="6" t="n">
-        <v>68291582</v>
-      </c>
-      <c r="F54" s="7" t="n">
-        <v>1.700633967936636</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="n"/>
-      <c r="B55" s="8" t="n"/>
-      <c r="C55" s="8" t="inlineStr">
+      <c r="D61" s="6" t="n">
+        <v>25813303</v>
+      </c>
+      <c r="E61" s="6" t="n">
+        <v>69773930</v>
+      </c>
+      <c r="F61" s="7" t="n">
+        <v>1.703022158768291</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="8" t="n"/>
+      <c r="B62" s="8" t="n"/>
+      <c r="C62" s="8" t="inlineStr">
         <is>
           <t>GDPPC</t>
         </is>
       </c>
-      <c r="D55" s="9" t="n">
-        <v>28779</v>
-      </c>
-      <c r="E55" s="9" t="n">
-        <v>38653.89</v>
-      </c>
-      <c r="F55" s="10" t="n">
-        <v>0.3431283227353278</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="11" t="inlineStr">
-        <is>
-          <t>Mitō</t>
-        </is>
-      </c>
-      <c r="B56" s="8" t="n">
-        <v>65</v>
-      </c>
-      <c r="C56" s="8" t="inlineStr">
+      <c r="D62" s="9" t="n">
+        <v>18360</v>
+      </c>
+      <c r="E62" s="9" t="n">
+        <v>26901</v>
+      </c>
+      <c r="F62" s="10" t="n">
+        <v>0.4651960784313726</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>Ralzawr</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>Area (km2)</t>
+        </is>
+      </c>
+      <c r="D63" s="6" t="n">
+        <v>871928.11</v>
+      </c>
+      <c r="E63" s="6" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="F63" s="7" t="n">
+        <v>0.7203253144344665</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="n"/>
+      <c r="B64" s="8" t="n"/>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>GDPPC</t>
+        </is>
+      </c>
+      <c r="D64" s="9" t="n">
+        <v>48800</v>
+      </c>
+      <c r="E64" s="9" t="n">
+        <v>58973</v>
+      </c>
+      <c r="F64" s="10" t="n">
+        <v>0.2084631147540984</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>Rhodellia</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="n">
+        <v>77</v>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
         <is>
           <t>Population</t>
         </is>
       </c>
-      <c r="D56" s="9" t="n">
-        <v>9723000</v>
-      </c>
-      <c r="E56" s="9" t="n">
-        <v>13723000</v>
-      </c>
-      <c r="F56" s="10" t="n">
-        <v>0.4113956597757893</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="4" t="inlineStr">
-        <is>
-          <t>Orioni</t>
-        </is>
-      </c>
-      <c r="B57" s="5" t="n">
-        <v>70</v>
-      </c>
-      <c r="C57" s="5" t="inlineStr">
+      <c r="D65" s="6" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="E65" s="6" t="n">
+        <v>24900000</v>
+      </c>
+      <c r="F65" s="7" t="n">
+        <v>1.49</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="n"/>
+      <c r="B66" s="8" t="n"/>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>GDPPC</t>
+        </is>
+      </c>
+      <c r="D66" s="9" t="n">
+        <v>45000</v>
+      </c>
+      <c r="E66" s="9" t="n">
+        <v>59500</v>
+      </c>
+      <c r="F66" s="10" t="n">
+        <v>0.3222222222222222</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>Sahra</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>Population</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="E67" s="6" t="n">
+        <v>40000000</v>
+      </c>
+      <c r="F67" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="n"/>
+      <c r="B68" s="8" t="n"/>
+      <c r="C68" s="8" t="inlineStr">
+        <is>
+          <t>GDPPC</t>
+        </is>
+      </c>
+      <c r="D68" s="9" t="n">
+        <v>10000</v>
+      </c>
+      <c r="E68" s="9" t="n">
+        <v>18000</v>
+      </c>
+      <c r="F68" s="10" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>Stedoria</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="n">
+        <v>86</v>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>Population</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="n">
+        <v>18727052</v>
+      </c>
+      <c r="E69" s="6" t="n">
+        <v>26409216</v>
+      </c>
+      <c r="F69" s="7" t="n">
+        <v>0.4102174757671416</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="n"/>
+      <c r="B70" s="8" t="n"/>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>GDPPC</t>
+        </is>
+      </c>
+      <c r="D70" s="9" t="n">
+        <v>14399</v>
+      </c>
+      <c r="E70" s="9" t="n">
+        <v>21161</v>
+      </c>
+      <c r="F70" s="10" t="n">
+        <v>0.4696159455517744</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>Sunseong</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="n">
+        <v>88</v>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>Population</t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="n">
+        <v>23660000</v>
+      </c>
+      <c r="E71" s="6" t="n">
+        <v>47600000</v>
+      </c>
+      <c r="F71" s="7" t="n">
+        <v>1.011834319526627</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="8" t="n"/>
+      <c r="B72" s="8" t="n"/>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>GDPPC</t>
+        </is>
+      </c>
+      <c r="D72" s="9" t="n">
+        <v>19369</v>
+      </c>
+      <c r="E72" s="9" t="n">
+        <v>29369</v>
+      </c>
+      <c r="F72" s="10" t="n">
+        <v>0.5162889152769891</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>Tagmatium</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="n">
+        <v>92</v>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
         <is>
           <t>Area (km2)</t>
         </is>
       </c>
-      <c r="D57" s="6" t="n">
-        <v>1155853</v>
-      </c>
-      <c r="E57" s="6" t="n">
-        <v>1320687</v>
-      </c>
-      <c r="F57" s="7" t="n">
-        <v>0.1426080998189216</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="8" t="n"/>
-      <c r="B58" s="8" t="n"/>
-      <c r="C58" s="8" t="inlineStr">
+      <c r="D73" s="6" t="n">
+        <v>1023597</v>
+      </c>
+      <c r="E73" s="6" t="n">
+        <v>1499825</v>
+      </c>
+      <c r="F73" s="7" t="n">
+        <v>0.4652495073744843</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="n"/>
+      <c r="B74" s="5" t="n"/>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>Population</t>
+        </is>
+      </c>
+      <c r="D74" s="6" t="n">
+        <v>253491524</v>
+      </c>
+      <c r="E74" s="6" t="n">
+        <v>274651624</v>
+      </c>
+      <c r="F74" s="7" t="n">
+        <v>0.08347458591948818</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="8" t="n"/>
+      <c r="B75" s="8" t="n"/>
+      <c r="C75" s="8" t="inlineStr">
         <is>
           <t>GDPPC</t>
         </is>
       </c>
-      <c r="D58" s="9" t="n">
-        <v>46131</v>
-      </c>
-      <c r="E58" s="9" t="n">
-        <v>58297.29</v>
-      </c>
-      <c r="F58" s="10" t="n">
-        <v>0.2637334980815504</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="4" t="inlineStr">
-        <is>
-          <t>Pentium</t>
-        </is>
-      </c>
-      <c r="B59" s="5" t="n">
-        <v>71</v>
-      </c>
-      <c r="C59" s="5" t="inlineStr">
+      <c r="D75" s="9" t="n">
+        <v>21595</v>
+      </c>
+      <c r="E75" s="9" t="n">
+        <v>37457</v>
+      </c>
+      <c r="F75" s="10" t="n">
+        <v>0.7345218800648298</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="11" t="inlineStr">
+        <is>
+          <t>Verraine</t>
+        </is>
+      </c>
+      <c r="B76" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="C76" s="8" t="inlineStr">
+        <is>
+          <t>Population</t>
+        </is>
+      </c>
+      <c r="D76" s="9" t="n">
+        <v>21072594</v>
+      </c>
+      <c r="E76" s="9" t="n">
+        <v>21000000</v>
+      </c>
+      <c r="F76" s="10" t="n">
+        <v>-0.003444948448207183</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>Volhynia</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="n">
+        <v>99</v>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
         <is>
           <t>Area (km2)</t>
         </is>
       </c>
-      <c r="D59" s="6" t="n">
-        <v>87500</v>
-      </c>
-      <c r="E59" s="6" t="n">
-        <v>389287</v>
-      </c>
-      <c r="F59" s="7" t="n">
-        <v>3.448994285714286</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="8" t="n"/>
-      <c r="B60" s="8" t="n"/>
-      <c r="C60" s="8" t="inlineStr">
+      <c r="D77" s="6" t="n">
+        <v>229900</v>
+      </c>
+      <c r="E77" s="6" t="n">
+        <v>94330</v>
+      </c>
+      <c r="F77" s="7" t="n">
+        <v>-0.5896911700739452</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="n"/>
+      <c r="B78" s="5" t="n"/>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>Population</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="n">
+        <v>16450000</v>
+      </c>
+      <c r="E78" s="6" t="n">
+        <v>12400000</v>
+      </c>
+      <c r="F78" s="7" t="n">
+        <v>-0.2462006079027356</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="8" t="n"/>
+      <c r="B79" s="8" t="n"/>
+      <c r="C79" s="8" t="inlineStr">
         <is>
           <t>GDPPC</t>
         </is>
       </c>
-      <c r="D60" s="9" t="n">
-        <v>21220</v>
-      </c>
-      <c r="E60" s="9" t="n">
-        <v>37542</v>
-      </c>
-      <c r="F60" s="10" t="n">
-        <v>0.7691800188501414</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="4" t="inlineStr">
-        <is>
-          <t>Poja</t>
-        </is>
-      </c>
-      <c r="B61" s="5" t="n">
-        <v>72</v>
-      </c>
-      <c r="C61" s="5" t="inlineStr">
+      <c r="D79" s="9" t="n">
+        <v>20000</v>
+      </c>
+      <c r="E79" s="9" t="n">
+        <v>23200</v>
+      </c>
+      <c r="F79" s="10" t="n">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>Welkija</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="n">
+        <v>102</v>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>Capital</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>Nowa Huta</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>Nowostolicna</t>
+        </is>
+      </c>
+      <c r="F80" s="5" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="n"/>
+      <c r="B81" s="5" t="n"/>
+      <c r="C81" s="5" t="inlineStr">
         <is>
           <t>Area (km2)</t>
         </is>
       </c>
-      <c r="D61" s="6" t="n">
-        <v>340090</v>
-      </c>
-      <c r="E61" s="6" t="n">
-        <v>504767</v>
-      </c>
-      <c r="F61" s="7" t="n">
-        <v>0.4842159428386604</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="5" t="n"/>
-      <c r="B62" s="5" t="n"/>
-      <c r="C62" s="5" t="inlineStr">
-        <is>
-          <t>Population</t>
-        </is>
-      </c>
-      <c r="D62" s="6" t="n">
-        <v>25813303</v>
-      </c>
-      <c r="E62" s="6" t="n">
-        <v>69773930</v>
-      </c>
-      <c r="F62" s="7" t="n">
-        <v>1.703022158768291</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="8" t="n"/>
-      <c r="B63" s="8" t="n"/>
-      <c r="C63" s="8" t="inlineStr">
-        <is>
-          <t>GDPPC</t>
-        </is>
-      </c>
-      <c r="D63" s="9" t="n">
-        <v>18360</v>
-      </c>
-      <c r="E63" s="9" t="n">
-        <v>26901</v>
-      </c>
-      <c r="F63" s="10" t="n">
-        <v>0.4651960784313726</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="4" t="inlineStr">
-        <is>
-          <t>Ralzawr</t>
-        </is>
-      </c>
-      <c r="B64" s="5" t="n">
-        <v>75</v>
-      </c>
-      <c r="C64" s="5" t="inlineStr">
-        <is>
-          <t>Area (km2)</t>
-        </is>
-      </c>
-      <c r="D64" s="6" t="n">
-        <v>871928.11</v>
-      </c>
-      <c r="E64" s="6" t="n">
-        <v>1500000</v>
-      </c>
-      <c r="F64" s="7" t="n">
-        <v>0.7203253144344665</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="8" t="n"/>
-      <c r="B65" s="8" t="n"/>
-      <c r="C65" s="8" t="inlineStr">
-        <is>
-          <t>GDPPC</t>
-        </is>
-      </c>
-      <c r="D65" s="9" t="n">
-        <v>48800</v>
-      </c>
-      <c r="E65" s="9" t="n">
-        <v>58973</v>
-      </c>
-      <c r="F65" s="10" t="n">
-        <v>0.2084631147540984</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="4" t="inlineStr">
-        <is>
-          <t>Rhodellia</t>
-        </is>
-      </c>
-      <c r="B66" s="5" t="n">
-        <v>77</v>
-      </c>
-      <c r="C66" s="5" t="inlineStr">
-        <is>
-          <t>Population</t>
-        </is>
-      </c>
-      <c r="D66" s="6" t="n">
-        <v>10000000</v>
-      </c>
-      <c r="E66" s="6" t="n">
-        <v>24900000</v>
-      </c>
-      <c r="F66" s="7" t="n">
-        <v>1.49</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="8" t="n"/>
-      <c r="B67" s="8" t="n"/>
-      <c r="C67" s="8" t="inlineStr">
-        <is>
-          <t>GDPPC</t>
-        </is>
-      </c>
-      <c r="D67" s="9" t="n">
-        <v>45000</v>
-      </c>
-      <c r="E67" s="9" t="n">
-        <v>59500</v>
-      </c>
-      <c r="F67" s="10" t="n">
-        <v>0.3222222222222222</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="4" t="inlineStr">
-        <is>
-          <t>Sahra</t>
-        </is>
-      </c>
-      <c r="B68" s="5" t="n">
-        <v>80</v>
-      </c>
-      <c r="C68" s="5" t="inlineStr">
-        <is>
-          <t>Population</t>
-        </is>
-      </c>
-      <c r="D68" s="6" t="n">
-        <v>20000000</v>
-      </c>
-      <c r="E68" s="6" t="n">
-        <v>40000000</v>
-      </c>
-      <c r="F68" s="7" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="8" t="n"/>
-      <c r="B69" s="8" t="n"/>
-      <c r="C69" s="8" t="inlineStr">
-        <is>
-          <t>GDPPC</t>
-        </is>
-      </c>
-      <c r="D69" s="9" t="n">
-        <v>10000</v>
-      </c>
-      <c r="E69" s="9" t="n">
-        <v>18000</v>
-      </c>
-      <c r="F69" s="10" t="n">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="4" t="inlineStr">
-        <is>
-          <t>Stedoria</t>
-        </is>
-      </c>
-      <c r="B70" s="5" t="n">
-        <v>86</v>
-      </c>
-      <c r="C70" s="5" t="inlineStr">
-        <is>
-          <t>Population</t>
-        </is>
-      </c>
-      <c r="D70" s="6" t="n">
-        <v>18727052</v>
-      </c>
-      <c r="E70" s="6" t="n">
-        <v>26409216</v>
-      </c>
-      <c r="F70" s="7" t="n">
-        <v>0.4102174757671416</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="8" t="n"/>
-      <c r="B71" s="8" t="n"/>
-      <c r="C71" s="8" t="inlineStr">
-        <is>
-          <t>GDPPC</t>
-        </is>
-      </c>
-      <c r="D71" s="9" t="n">
-        <v>14399</v>
-      </c>
-      <c r="E71" s="9" t="n">
-        <v>21161</v>
-      </c>
-      <c r="F71" s="10" t="n">
-        <v>0.4696159455517744</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="4" t="inlineStr">
-        <is>
-          <t>Sunseong</t>
-        </is>
-      </c>
-      <c r="B72" s="5" t="n">
-        <v>88</v>
-      </c>
-      <c r="C72" s="5" t="inlineStr">
-        <is>
-          <t>Population</t>
-        </is>
-      </c>
-      <c r="D72" s="6" t="n">
-        <v>23660000</v>
-      </c>
-      <c r="E72" s="6" t="n">
-        <v>47600000</v>
-      </c>
-      <c r="F72" s="7" t="n">
-        <v>1.011834319526627</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="8" t="n"/>
-      <c r="B73" s="8" t="n"/>
-      <c r="C73" s="8" t="inlineStr">
-        <is>
-          <t>GDPPC</t>
-        </is>
-      </c>
-      <c r="D73" s="9" t="n">
-        <v>19369</v>
-      </c>
-      <c r="E73" s="9" t="n">
-        <v>29369</v>
-      </c>
-      <c r="F73" s="10" t="n">
-        <v>0.5162889152769891</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="4" t="inlineStr">
-        <is>
-          <t>Tagmatium</t>
-        </is>
-      </c>
-      <c r="B74" s="5" t="n">
-        <v>92</v>
-      </c>
-      <c r="C74" s="5" t="inlineStr">
-        <is>
-          <t>Area (km2)</t>
-        </is>
-      </c>
-      <c r="D74" s="6" t="n">
-        <v>1023597</v>
-      </c>
-      <c r="E74" s="6" t="n">
-        <v>1499825</v>
-      </c>
-      <c r="F74" s="7" t="n">
-        <v>0.4652495073744843</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="5" t="n"/>
-      <c r="B75" s="5" t="n"/>
-      <c r="C75" s="5" t="inlineStr">
-        <is>
-          <t>Population</t>
-        </is>
-      </c>
-      <c r="D75" s="6" t="n">
-        <v>253491524</v>
-      </c>
-      <c r="E75" s="6" t="n">
-        <v>274651624</v>
-      </c>
-      <c r="F75" s="7" t="n">
-        <v>0.08347458591948818</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="8" t="n"/>
-      <c r="B76" s="8" t="n"/>
-      <c r="C76" s="8" t="inlineStr">
-        <is>
-          <t>GDPPC</t>
-        </is>
-      </c>
-      <c r="D76" s="9" t="n">
-        <v>21595</v>
-      </c>
-      <c r="E76" s="9" t="n">
-        <v>37457</v>
-      </c>
-      <c r="F76" s="10" t="n">
-        <v>0.7345218800648298</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="11" t="inlineStr">
-        <is>
-          <t>Verraine</t>
-        </is>
-      </c>
-      <c r="B77" s="8" t="n">
-        <v>98</v>
-      </c>
-      <c r="C77" s="8" t="inlineStr">
-        <is>
-          <t>Population</t>
-        </is>
-      </c>
-      <c r="D77" s="9" t="n">
-        <v>21072594</v>
-      </c>
-      <c r="E77" s="9" t="n">
-        <v>21000000</v>
-      </c>
-      <c r="F77" s="10" t="n">
-        <v>-0.003444948448207183</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="4" t="inlineStr">
-        <is>
-          <t>Volhynia</t>
-        </is>
-      </c>
-      <c r="B78" s="5" t="n">
-        <v>99</v>
-      </c>
-      <c r="C78" s="5" t="inlineStr">
-        <is>
-          <t>Area (km2)</t>
-        </is>
-      </c>
-      <c r="D78" s="6" t="n">
-        <v>229900</v>
-      </c>
-      <c r="E78" s="6" t="n">
-        <v>94330</v>
-      </c>
-      <c r="F78" s="7" t="n">
-        <v>-0.5896911700739452</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="5" t="n"/>
-      <c r="B79" s="5" t="n"/>
-      <c r="C79" s="5" t="inlineStr">
-        <is>
-          <t>Population</t>
-        </is>
-      </c>
-      <c r="D79" s="6" t="n">
-        <v>16450000</v>
-      </c>
-      <c r="E79" s="6" t="n">
-        <v>12400000</v>
-      </c>
-      <c r="F79" s="7" t="n">
-        <v>-0.2462006079027356</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="8" t="n"/>
-      <c r="B80" s="8" t="n"/>
-      <c r="C80" s="8" t="inlineStr">
-        <is>
-          <t>GDPPC</t>
-        </is>
-      </c>
-      <c r="D80" s="9" t="n">
-        <v>20000</v>
-      </c>
-      <c r="E80" s="9" t="n">
-        <v>23200</v>
-      </c>
-      <c r="F80" s="10" t="n">
-        <v>0.16</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="4" t="inlineStr">
-        <is>
-          <t>Welkija</t>
-        </is>
-      </c>
-      <c r="B81" s="5" t="n">
-        <v>102</v>
-      </c>
-      <c r="C81" s="5" t="inlineStr">
-        <is>
-          <t>Capital</t>
-        </is>
-      </c>
-      <c r="D81" s="5" t="inlineStr">
-        <is>
-          <t>Nowa Huta</t>
-        </is>
-      </c>
-      <c r="E81" s="5" t="inlineStr">
-        <is>
-          <t>Nowostolicna</t>
-        </is>
-      </c>
-      <c r="F81" s="5" t="n"/>
+      <c r="D81" s="6" t="n">
+        <v>650602</v>
+      </c>
+      <c r="E81" s="6" t="n">
+        <v>650000</v>
+      </c>
+      <c r="F81" s="7" t="n">
+        <v>-0.0009252968788906274</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="n"/>
       <c r="B82" s="5" t="n"/>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>Area (km2)</t>
+          <t>Population</t>
         </is>
       </c>
       <c r="D82" s="6" t="n">
-        <v>650602</v>
+        <v>14263654</v>
       </c>
       <c r="E82" s="6" t="n">
-        <v>650000</v>
+        <v>40000000</v>
       </c>
       <c r="F82" s="7" t="n">
-        <v>-0.0009252968788906274</v>
+        <v>1.804330503249728</v>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="5" t="n"/>
-      <c r="B83" s="5" t="n"/>
-      <c r="C83" s="5" t="inlineStr">
+      <c r="A83" s="8" t="n"/>
+      <c r="B83" s="8" t="n"/>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t>GDPPC</t>
+        </is>
+      </c>
+      <c r="D83" s="9" t="n">
+        <v>14126</v>
+      </c>
+      <c r="E83" s="9" t="n">
+        <v>26000</v>
+      </c>
+      <c r="F83" s="10" t="n">
+        <v>0.8405776582188872</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>Ymutz-Mizlan</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="n">
+        <v>105</v>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
         <is>
           <t>Population</t>
         </is>
       </c>
-      <c r="D83" s="6" t="n">
-        <v>14263654</v>
-      </c>
-      <c r="E83" s="6" t="n">
-        <v>40000000</v>
-      </c>
-      <c r="F83" s="7" t="n">
-        <v>1.804330503249728</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="8" t="n"/>
-      <c r="B84" s="8" t="n"/>
-      <c r="C84" s="8" t="inlineStr">
+      <c r="D84" s="6" t="n">
+        <v>30203486</v>
+      </c>
+      <c r="E84" s="6" t="n">
+        <v>60000000</v>
+      </c>
+      <c r="F84" s="7" t="n">
+        <v>0.9865256613094263</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="8" t="n"/>
+      <c r="B85" s="8" t="n"/>
+      <c r="C85" s="8" t="inlineStr">
         <is>
           <t>GDPPC</t>
         </is>
       </c>
-      <c r="D84" s="9" t="n">
-        <v>14126</v>
-      </c>
-      <c r="E84" s="9" t="n">
-        <v>26000</v>
-      </c>
-      <c r="F84" s="10" t="n">
-        <v>0.8405776582188872</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="4" t="inlineStr">
-        <is>
-          <t>Ymutz-Mizlan</t>
-        </is>
-      </c>
-      <c r="B85" s="5" t="n">
-        <v>105</v>
-      </c>
-      <c r="C85" s="5" t="inlineStr">
-        <is>
-          <t>Population</t>
-        </is>
-      </c>
-      <c r="D85" s="6" t="n">
-        <v>30203486</v>
-      </c>
-      <c r="E85" s="6" t="n">
-        <v>60000000</v>
-      </c>
-      <c r="F85" s="7" t="n">
-        <v>0.9865256613094263</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="8" t="n"/>
-      <c r="B86" s="8" t="n"/>
-      <c r="C86" s="8" t="inlineStr">
-        <is>
-          <t>GDPPC</t>
-        </is>
-      </c>
-      <c r="D86" s="9" t="n">
+      <c r="D85" s="9" t="n">
         <v>7000</v>
       </c>
-      <c r="E86" s="9" t="n">
+      <c r="E85" s="9" t="n">
         <v>15000</v>
       </c>
-      <c r="F86" s="10" t="n">
+      <c r="F85" s="10" t="n">
         <v>1.142857142857143</v>
       </c>
     </row>
-    <row r="87"/>
+    <row r="86"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:F2"/>
@@ -3982,8 +3958,8 @@
       <c r="C59" s="6" t="n">
         <v>339988.16</v>
       </c>
-      <c r="D59" s="13" t="n">
-        <v>361225</v>
+      <c r="D59" s="6" t="n">
+        <v>18361225</v>
       </c>
       <c r="E59" s="6" t="n">
         <v>20092</v>

</xml_diff>